<commit_message>
deja cambiarme de rama
</commit_message>
<xml_diff>
--- a/data/DCH/160kW_2dias/elmo_data.xlsx
+++ b/data/DCH/160kW_2dias/elmo_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TECNO-MASTER\Desktop\Elmo_infrastructure_sizing_NP-\data\DCH\160kW_2dias\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9C37A4B-1AA3-42E0-A0C8-CA630C325810}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B004FD3-20B7-457F-93EC-9F00C8EFF2E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LHD" sheetId="2" r:id="rId1"/>
@@ -3248,6 +3248,7 @@
     <col min="4" max="4" width="14.140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="16.140625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>